<commit_message>
docs(artigo): revise title, add references and recompute Likert chart
- artigo-movy.tex: update title to emphasize prototypal implementation;
  add xurl/longtable packages and URL breaking for the bibliography
- referencias.bib: add IBGE REGIC, Silva (2022) and Bizerril (2024)
  references; adjust thesis types and author casing
- gerar-grafico-likert.py: keep all 19 responses (only open answers of
  response 11 were discarded, closed Likert items remain valid)
- update responses spreadsheet and regenerate grafico-likert.png
- add reference notes (refes/) and Cloudflare Workers deploy log

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/artigo/Avaliação exploratória do sistema Movy (respostas).xlsx
+++ b/docs/artigo/Avaliação exploratória do sistema Movy (respostas).xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="298" uniqueCount="107">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="425" uniqueCount="133">
   <si>
     <t>Carimbo de data/hora</t>
   </si>
@@ -342,6 +342,84 @@
   </si>
   <si>
     <t>Não se aplica</t>
+  </si>
+  <si>
+    <t>A praticidade de organizar.</t>
+  </si>
+  <si>
+    <t>Confundi-me sobre as "paradas". Imaginei que seriam os locais onde o transporte pararia durante a viagem, a fim de permitir que os passageiros realizassem suas necessidades fisiológicas.</t>
+  </si>
+  <si>
+    <t>Por ser um sistema direcionado à viagens, possui ampla funcionalidade para essa finalidade. Há maior organização.</t>
+  </si>
+  <si>
+    <t>Muito bom!</t>
+  </si>
+  <si>
+    <t>A mostragem de todas as viagens disponíveis, facilitando a procura e escolha.</t>
+  </si>
+  <si>
+    <t>Nada.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Não. </t>
+  </si>
+  <si>
+    <t>Nenhuma.</t>
+  </si>
+  <si>
+    <t>Sim, porque oferece um serviço rápido e eficaz.</t>
+  </si>
+  <si>
+    <t>Lacrou!</t>
+  </si>
+  <si>
+    <t>Parcialmente</t>
+  </si>
+  <si>
+    <t>Tudo</t>
+  </si>
+  <si>
+    <t>Nada</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Não </t>
+  </si>
+  <si>
+    <t xml:space="preserve">. </t>
+  </si>
+  <si>
+    <t>Rapido</t>
+  </si>
+  <si>
+    <t>Bom!</t>
+  </si>
+  <si>
+    <t>Fácil de usar e entender.</t>
+  </si>
+  <si>
+    <t>Não!</t>
+  </si>
+  <si>
+    <t>Não visualizei nenhum defeito no meu ponto de vista.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mais organizado </t>
+  </si>
+  <si>
+    <t>Bom!!!</t>
+  </si>
+  <si>
+    <t>A facilidade de cadastrar os dados e por em prática as ações.</t>
+  </si>
+  <si>
+    <t>Alterar as "paradas" para "parada de embarque" e "parada de desembarque".</t>
+  </si>
+  <si>
+    <t>Sim. É nem mais prático.</t>
+  </si>
+  <si>
+    <t>Está ótimo</t>
   </si>
 </sst>
 </file>
@@ -482,7 +560,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:AJ14" displayName="Form_Responses" name="Form_Responses" id="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:AJ20" displayName="Form_Responses" name="Form_Responses" id="1">
   <tableColumns count="36">
     <tableColumn name="Carimbo de data/hora" id="1"/>
     <tableColumn name="Você é estudante universitário?  " id="2"/>
@@ -1717,6 +1795,417 @@
         <v>46</v>
       </c>
     </row>
+    <row r="15" ht="22.5" customHeight="1">
+      <c r="A15" s="6">
+        <v>46212.496837743056</v>
+      </c>
+      <c r="B15" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="C15" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="D15" s="7" t="s">
+        <v>71</v>
+      </c>
+      <c r="I15" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="J15" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="K15" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="L15" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="M15" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="N15" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="V15" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="W15" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="X15" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="Y15" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="Z15" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="AA15" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="AB15" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="AC15" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="AD15" s="7" t="s">
+        <v>107</v>
+      </c>
+      <c r="AE15" s="7" t="s">
+        <v>108</v>
+      </c>
+      <c r="AF15" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="AH15" s="7" t="s">
+        <v>109</v>
+      </c>
+      <c r="AI15" s="7" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="16" ht="22.5" customHeight="1">
+      <c r="A16" s="6">
+        <v>46212.50410229167</v>
+      </c>
+      <c r="B16" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="C16" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="D16" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="E16" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="F16" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="G16" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="H16" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="V16" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="W16" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="X16" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="Y16" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="Z16" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="AA16" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="AB16" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="AC16" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="AD16" s="7" t="s">
+        <v>111</v>
+      </c>
+      <c r="AE16" s="7" t="s">
+        <v>112</v>
+      </c>
+      <c r="AF16" s="7" t="s">
+        <v>113</v>
+      </c>
+      <c r="AG16" s="7" t="s">
+        <v>114</v>
+      </c>
+      <c r="AH16" s="7" t="s">
+        <v>115</v>
+      </c>
+      <c r="AI16" s="7" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="17" ht="22.5" customHeight="1">
+      <c r="A17" s="6">
+        <v>46212.567322939816</v>
+      </c>
+      <c r="B17" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="C17" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="D17" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="E17" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="F17" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="G17" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="H17" s="7" t="s">
+        <v>117</v>
+      </c>
+      <c r="V17" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="W17" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="X17" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="Y17" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="Z17" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="AA17" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="AB17" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="AC17" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="AD17" s="7" t="s">
+        <v>118</v>
+      </c>
+      <c r="AE17" s="7" t="s">
+        <v>119</v>
+      </c>
+      <c r="AF17" s="7" t="s">
+        <v>120</v>
+      </c>
+      <c r="AG17" s="7" t="s">
+        <v>121</v>
+      </c>
+      <c r="AH17" s="7" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="18" ht="22.5" customHeight="1">
+      <c r="A18" s="6">
+        <v>46212.57809271991</v>
+      </c>
+      <c r="B18" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="C18" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="D18" s="7" t="s">
+        <v>71</v>
+      </c>
+      <c r="I18" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="J18" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="K18" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="L18" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="M18" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="N18" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="V18" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="W18" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="X18" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="Y18" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="Z18" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="AA18" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="AB18" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="AC18" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="AD18" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="AE18" s="7" t="s">
+        <v>120</v>
+      </c>
+      <c r="AF18" s="7" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="19" ht="22.5" customHeight="1">
+      <c r="A19" s="6">
+        <v>46212.694780624995</v>
+      </c>
+      <c r="B19" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="C19" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="D19" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="E19" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="F19" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="G19" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="H19" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="V19" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="W19" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="X19" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="Y19" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="Z19" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="AA19" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="AB19" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="AC19" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="AD19" s="7" t="s">
+        <v>123</v>
+      </c>
+      <c r="AE19" s="7" t="s">
+        <v>124</v>
+      </c>
+      <c r="AF19" s="7" t="s">
+        <v>125</v>
+      </c>
+      <c r="AG19" s="7" t="s">
+        <v>126</v>
+      </c>
+      <c r="AH19" s="7" t="s">
+        <v>127</v>
+      </c>
+      <c r="AI19" s="7" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="20" ht="22.5" customHeight="1">
+      <c r="A20" s="6">
+        <v>46212.73794579861</v>
+      </c>
+      <c r="B20" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="C20" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="D20" s="7" t="s">
+        <v>71</v>
+      </c>
+      <c r="I20" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="J20" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="K20" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="L20" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="M20" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="N20" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="V20" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="W20" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="X20" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="Y20" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="Z20" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="AA20" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="AB20" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="AC20" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="AD20" s="7" t="s">
+        <v>129</v>
+      </c>
+      <c r="AE20" s="7" t="s">
+        <v>112</v>
+      </c>
+      <c r="AF20" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="AG20" s="7" t="s">
+        <v>130</v>
+      </c>
+      <c r="AH20" s="7" t="s">
+        <v>131</v>
+      </c>
+      <c r="AI20" s="7" t="s">
+        <v>132</v>
+      </c>
+    </row>
   </sheetData>
   <drawing r:id="rId1"/>
   <tableParts count="1">

</xml_diff>